<commit_message>
Trazabilidad: Corrección matriz RFvsCU acorde a los casos de uso actuales.
</commit_message>
<xml_diff>
--- a/Documento 0/Matriz_RF_vs_CU.xlsx
+++ b/Documento 0/Matriz_RF_vs_CU.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="106">
   <si>
     <t>CU1</t>
   </si>
@@ -945,7 +945,9 @@
       <c r="AT3" s="1"/>
       <c r="AU3" s="1"/>
       <c r="AV3" s="1"/>
-      <c r="AW3" s="1"/>
+      <c r="AW3" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="AX3" s="1"/>
       <c r="AY3" s="1"/>
       <c r="AZ3" s="1"/>
@@ -992,11 +994,15 @@
       <c r="AB4" s="1"/>
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
-      <c r="AE4" s="1"/>
+      <c r="AE4" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="1"/>
-      <c r="AI4" s="1"/>
+      <c r="AI4" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="8" t="s">
         <v>53</v>
@@ -2305,9 +2311,7 @@
       <c r="AB25" s="1"/>
       <c r="AC25" s="1"/>
       <c r="AD25" s="1"/>
-      <c r="AE25" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="AE25" s="1"/>
       <c r="AF25" s="1"/>
       <c r="AG25" s="1"/>
       <c r="AH25" s="1"/>
@@ -2327,9 +2331,7 @@
       <c r="AT25" s="1"/>
       <c r="AU25" s="1"/>
       <c r="AV25" s="1"/>
-      <c r="AW25" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="AW25" s="1"/>
       <c r="AX25" s="1"/>
       <c r="AY25" s="1"/>
       <c r="AZ25" s="1"/>
@@ -2368,9 +2370,7 @@
       <c r="AB26" s="1"/>
       <c r="AC26" s="1"/>
       <c r="AD26" s="1"/>
-      <c r="AE26" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="AE26" s="1"/>
       <c r="AF26" s="1"/>
       <c r="AG26" s="1"/>
       <c r="AH26" s="1"/>
@@ -2511,7 +2511,9 @@
       <c r="AS28" s="1"/>
       <c r="AT28" s="1"/>
       <c r="AU28" s="1"/>
-      <c r="AV28" s="1"/>
+      <c r="AV28" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="AW28" s="1"/>
       <c r="AX28" s="1"/>
       <c r="AY28" s="1"/>
@@ -2551,9 +2553,7 @@
       <c r="AB29" s="1"/>
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
-      <c r="AE29" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="AE29" s="1"/>
       <c r="AF29" s="1"/>
       <c r="AG29" s="1"/>
       <c r="AH29" s="1"/>
@@ -2610,9 +2610,7 @@
       <c r="AB30" s="1"/>
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
-      <c r="AE30" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="AE30" s="1"/>
       <c r="AF30" s="1"/>
       <c r="AG30" s="1"/>
       <c r="AH30" s="1"/>
@@ -2854,9 +2852,7 @@
       <c r="AF34" s="1"/>
       <c r="AG34" s="1"/>
       <c r="AH34" s="1"/>
-      <c r="AI34" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="AI34" s="1"/>
       <c r="AJ34" s="1"/>
       <c r="AK34" s="1"/>
       <c r="AL34" s="1"/>

</xml_diff>